<commit_message>
Add procurement cost disclaimer
</commit_message>
<xml_diff>
--- a/docs/MECHANICAL_PROCUREMENT_LIST.xlsx
+++ b/docs/MECHANICAL_PROCUREMENT_LIST.xlsx
@@ -3771,8 +3771,8 @@
           <t>采购执行概览</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="56" t="inlineStr">
@@ -3901,8 +3901,8 @@
           <t>是：已采购</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3910,8 +3910,8 @@
           <t>默认整车加工配置：纯惯导车模 v4.0.3、加强茎 v7.0.0、1:5 齿轮 v1.3.1。</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -3919,8 +3919,6 @@
           <t>光电管车模、1:8.5 齿轮和电磁支架已标为可选，不应与默认版本重复下单。</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -3928,8 +3926,6 @@
           <t>CNC 加工要求：所有需螺丝固定的 CNC 件必须按图增加 M2 螺纹孔，不能只留光孔；加工后逐孔试装确认。</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -3937,8 +3933,6 @@
           <t>加工购买方式：边板/侧板搜“铨洲”；车模/加强茎搜“哈长伟”；齿轮由嘉立创按 PA12S 打印；粘胶和电磁支架自行 3D 打印。</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3946,8 +3940,6 @@
           <t>链接核验说明：2026-08-27 已通过淘宝商品详情页核验；“有货/预售”仅代表核验时页面状态，最终以下单页为准。</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Add encoder magnet to procurement list
</commit_message>
<xml_diff>
--- a/docs/MECHANICAL_PROCUREMENT_LIST.xlsx
+++ b/docs/MECHANICAL_PROCUREMENT_LIST.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'采购清单'!$A$4:$L$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'采购清单'!$A$4:$L$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'采购清单'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -572,7 +572,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -725,6 +725,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00D6B656"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
@@ -874,7 +880,7 @@
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -1070,6 +1076,13 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
+    <xf numFmtId="0" fontId="35" fillId="42" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="54" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1219,8 +1232,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProcurementList" displayName="ProcurementList" ref="A4:L44" headerRowCount="1">
-  <autoFilter ref="A4:L44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProcurementList" displayName="ProcurementList" ref="A4:L45" headerRowCount="1">
+  <autoFilter ref="A4:L45"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="类别"/>
@@ -1527,7 +1540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1628,2115 +1641,2116 @@
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="13" t="n">
+      <c r="A5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>CNC 加工</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>主支撑加强筋</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>加强茎 v7.0.0；2 份</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>碳纤维板</t>
         </is>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="13" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>纯惯导版本必做。原文件名“加强茎”沿用建模命名。 CNC 必须按图增加 M2 螺纹孔，并逐孔试装确认。</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J5" s="14" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>淘宝搜索“哈长伟”；按 STEP 文件 CNC 加工</t>
         </is>
       </c>
-      <c r="K5" s="14" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>mechanical/step/加强茎v7.0.0.STEP</t>
         </is>
       </c>
-      <c r="L5" s="14" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="15" t="n">
+      <c r="A6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>CNC 加工</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>侧板 / 电机支撑</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>侧板 v3.2.6；2 份</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>碳纤维板</t>
         </is>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H6" s="16" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>必做；电机支撑。以 STEP 文件为加工依据。 CNC 必须按图增加 M2 螺纹孔，并逐孔试装确认。</t>
         </is>
       </c>
-      <c r="I6" s="15" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J6" s="16" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>浏览器搜索“铨洲”；按 STEP 文件 CNC 加工</t>
         </is>
       </c>
-      <c r="K6" s="16" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>mechanical/step/侧板v3.2.6.STEP</t>
         </is>
       </c>
-      <c r="L6" s="16" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="15" t="n">
+      <c r="A7" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>CNC 加工</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>纯惯导车模底板</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>车模 v4.0.3；1 份</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>碳纤维板</t>
         </is>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>纯惯导版本必做；搭配加强茎 v7.0.0。以 STEP 文件为加工依据。 CNC 必须按图增加 M2 螺纹孔，并逐孔试装确认。</t>
         </is>
       </c>
-      <c r="I7" s="15" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J7" s="16" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>淘宝搜索“哈长伟”；按 STEP 文件 CNC 加工</t>
         </is>
       </c>
-      <c r="K7" s="16" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>mechanical/step/车模v4.0.3.STEP</t>
         </is>
       </c>
-      <c r="L7" s="16" t="inlineStr"/>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="15" t="n">
+      <c r="A8" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>CNC 加工</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>边板 / 轮毂支撑</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>边板2 v2.3.5；2 份</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>碳纤维板</t>
         </is>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>必做；轮毂支撑。以 STEP 文件为加工依据。 CNC 必须按图增加 M2 螺纹孔，并逐孔试装确认。</t>
         </is>
       </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J8" s="16" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>浏览器搜索“铨洲”；按 STEP 文件 CNC 加工</t>
         </is>
       </c>
-      <c r="K8" s="16" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>mechanical/step/边板2v2.3.5.STEP</t>
         </is>
       </c>
-      <c r="L8" s="16" t="inlineStr"/>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="17" t="n">
+      <c r="A9" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>3D 打印</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>轮毂齿轮</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>齿轮 v1.3.1；1:5 减速比；配套小齿轮为 0.5 模 10 齿；2 份</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>PA12S</t>
         </is>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>纯惯导当前 1:5 配置；推荐嘉立创 PA12S。</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J9" s="18" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>嘉立创 3D 打印 PA12S；上传对应 STEP 文件</t>
         </is>
       </c>
-      <c r="K9" s="18" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>mechanical/step/齿轮v1.3.1.STEP</t>
         </is>
       </c>
-      <c r="L9" s="18" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>与 0.5 模 10 齿黄铜小齿轮配套。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="19" t="n">
+      <c r="A10" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>3D 打印</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>磁铁固定件</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>粘胶 v7；2 份</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>PLA + PETG</t>
         </is>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>必做；原说明建议 PLA 与 PETG 双料打印。</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J10" s="20" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>自行 3D 打印；建议 PLA + PETG 双料打印</t>
         </is>
       </c>
-      <c r="K10" s="20" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>mechanical/step/粘胶v7.STEP</t>
         </is>
       </c>
-      <c r="L10" s="20" t="inlineStr"/>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="21" t="n">
+      <c r="A11" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>可选 CNC 加工</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>光电管版本加强筋</t>
         </is>
       </c>
-      <c r="D11" s="22" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>加强茎 v6.1.1；2 份</t>
         </is>
       </c>
-      <c r="E11" s="22" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>碳纤维板</t>
         </is>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="21" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H11" s="22" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>光电管车模版本；与纯惯导 v7.0.0 二选一。 CNC 必须按图增加 M2 螺纹孔，并逐孔试装确认。</t>
         </is>
       </c>
-      <c r="I11" s="21" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J11" s="22" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>淘宝搜索“哈长伟”；按 STEP 文件 CNC 加工</t>
         </is>
       </c>
-      <c r="K11" s="22" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>mechanical/step/加强茎v6.1.1.STEP</t>
         </is>
       </c>
-      <c r="L11" s="22" t="inlineStr"/>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="23" t="n">
+      <c r="A12" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>可选 CNC 加工</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>光电管车模底板</t>
         </is>
       </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>车模 v3.9.5；1 份</t>
         </is>
       </c>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>碳纤维板</t>
         </is>
       </c>
-      <c r="F12" s="23" t="n">
+      <c r="F12" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="23" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H12" s="24" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>光电管车模版本；与纯惯导 v4.0.3 二选一，搭配加强茎 v6.1.1。 CNC 必须按图增加 M2 螺纹孔，并逐孔试装确认。</t>
         </is>
       </c>
-      <c r="I12" s="23" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>淘宝搜索“哈长伟”；按 STEP 文件 CNC 加工</t>
         </is>
       </c>
-      <c r="K12" s="24" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>mechanical/step/车模v3.9.5.STEP</t>
         </is>
       </c>
-      <c r="L12" s="24" t="inlineStr"/>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="25" t="n">
+      <c r="A13" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>可选 3D 打印</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>轮毂齿轮</t>
         </is>
       </c>
-      <c r="D13" s="26" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>齿轮 v1.1.4；1:8.5 减速比；配套小齿轮为 0.4 模 8 齿；2 份</t>
         </is>
       </c>
-      <c r="E13" s="26" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>PA12S</t>
         </is>
       </c>
-      <c r="F13" s="25" t="n">
+      <c r="F13" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="25" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H13" s="26" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>普通 1:8.5 配置；与 1:5 齿轮二选一。</t>
         </is>
       </c>
-      <c r="I13" s="25" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J13" s="26" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>嘉立创 3D 打印 PA12S；上传对应 STEP 文件</t>
         </is>
       </c>
-      <c r="K13" s="26" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>mechanical/step/齿轮v1.1.4.STEP</t>
         </is>
       </c>
-      <c r="L13" s="26" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>与 0.4 模 8 齿黄铜小齿轮配套。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="27" t="n">
+      <c r="A14" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>可选 3D 打印</t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>电磁支架（方案 A）</t>
         </is>
       </c>
-      <c r="D14" s="28" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>电磁支架 v1.0.0</t>
         </is>
       </c>
-      <c r="E14" s="28" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>PLA</t>
         </is>
       </c>
-      <c r="F14" s="27" t="n">
+      <c r="F14" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="27" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H14" s="28" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>仅电磁组需要，不属于纯惯导整车必做件。</t>
         </is>
       </c>
-      <c r="I14" s="27" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J14" s="28" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>自行 3D 打印 PLA</t>
         </is>
       </c>
-      <c r="K14" s="28" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>mechanical/step/电磁支架v1.0.0.STEP</t>
         </is>
       </c>
-      <c r="L14" s="28" t="inlineStr"/>
     </row>
     <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="27" t="n">
+      <c r="A15" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>可选 3D 打印</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>电磁支架（方案 B）</t>
         </is>
       </c>
-      <c r="D15" s="28" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>电磁支架2 v1.0.0</t>
         </is>
       </c>
-      <c r="E15" s="28" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>PLA</t>
         </is>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="27" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H15" s="28" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>仅电磁组需要；与方案 A 二选一。</t>
         </is>
       </c>
-      <c r="I15" s="27" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J15" s="28" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>自行 3D 打印 PLA</t>
         </is>
       </c>
-      <c r="K15" s="28" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>mechanical/step/电磁支架2v1.0.0.STEP</t>
         </is>
       </c>
-      <c r="L15" s="28" t="inlineStr"/>
     </row>
     <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="29" t="n">
+      <c r="A16" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="30" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C16" s="30" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>平垫片</t>
         </is>
       </c>
-      <c r="D16" s="30" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="E16" s="30" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>PEEK</t>
         </is>
       </c>
-      <c r="F16" s="29" t="n">
+      <c r="F16" t="n">
         <v>10</v>
       </c>
-      <c r="G16" s="29" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>片</t>
         </is>
       </c>
-      <c r="H16" s="30" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>下单选 M2【10个】。</t>
         </is>
       </c>
-      <c r="I16" s="29" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J16" s="31" t="inlineStr">
+      <c r="J16" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mcCPRhR8r6Abf2?tk=67dST3um0aT</t>
         </is>
       </c>
-      <c r="K16" s="30" t="n"/>
-      <c r="L16" s="30" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>已核验：在售、有货；包装数匹配。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="32" t="n">
+      <c r="A17" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="33" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C17" s="33" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>平垫片</t>
         </is>
       </c>
-      <c r="D17" s="33" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>M2.5</t>
         </is>
       </c>
-      <c r="E17" s="33" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>PEEK</t>
         </is>
       </c>
-      <c r="F17" s="32" t="n">
+      <c r="F17" t="n">
         <v>10</v>
       </c>
-      <c r="G17" s="32" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>片</t>
         </is>
       </c>
-      <c r="H17" s="33" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>下单选 M2.5【10个】。</t>
         </is>
       </c>
-      <c r="I17" s="32" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J17" s="34" t="inlineStr">
+      <c r="J17" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mcCPRhR8r6Abf2?tk=67dST3um0aT</t>
         </is>
       </c>
-      <c r="K17" s="33" t="n"/>
-      <c r="L17" s="33" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>已核验：在售、有货；包装数匹配。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="32" t="n">
+      <c r="A18" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="33" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>盘头螺丝</t>
         </is>
       </c>
-      <c r="D18" s="33" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>M2 x 10 mm</t>
         </is>
       </c>
-      <c r="E18" s="33" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>PEEK</t>
         </is>
       </c>
-      <c r="F18" s="32" t="n">
+      <c r="F18" t="n">
         <v>4</v>
       </c>
-      <c r="G18" s="32" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H18" s="33" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>需要 4 颗；下单选 M2*10，按单价购买 4 颗。</t>
         </is>
       </c>
-      <c r="I18" s="32" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J18" s="34" t="inlineStr">
+      <c r="J18" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8k9zIJYJO9kp8Hs?tk=jm5VT3ulzzo</t>
         </is>
       </c>
-      <c r="K18" s="33" t="n"/>
-      <c r="L18" s="33" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>已核验：在售、有货。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="32" t="n">
+      <c r="A19" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="33" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>螺丝</t>
         </is>
       </c>
-      <c r="D19" s="33" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>M2.5 x 6 mm</t>
         </is>
       </c>
-      <c r="E19" s="33" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>PEEK</t>
         </is>
       </c>
-      <c r="F19" s="32" t="n">
+      <c r="F19" t="n">
         <v>8</v>
       </c>
-      <c r="G19" s="32" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H19" s="33" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>需要 8 颗；下单选 M2.5*6[2只]，下单数量选 4。</t>
         </is>
       </c>
-      <c r="I19" s="32" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J19" s="34" t="inlineStr">
+      <c r="J19" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mcyAufcbGLKcY3?tk=XZ90T3unac3</t>
         </is>
       </c>
-      <c r="K19" s="33" t="n"/>
-      <c r="L19" s="33" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>已核验：在售、有货。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="32" t="n">
+      <c r="A20" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="33" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>螺母</t>
         </is>
       </c>
-      <c r="D20" s="33" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="E20" s="33" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>PEEK</t>
         </is>
       </c>
-      <c r="F20" s="32" t="n">
+      <c r="F20" t="n">
         <v>4</v>
       </c>
-      <c r="G20" s="32" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H20" s="33" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>需要 4 颗；商品为 M2【2只】，下单数量选 2。</t>
         </is>
       </c>
-      <c r="I20" s="32" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J20" s="34" t="inlineStr">
+      <c r="J20" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mczamPgTZqUGx8?tk=T7OHT3uNCEz</t>
         </is>
       </c>
-      <c r="K20" s="33" t="n"/>
-      <c r="L20" s="33" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>已核验：在售、有货。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1">
-      <c r="A21" s="32" t="n">
+      <c r="A21" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="33" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C21" s="33" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>垫片</t>
         </is>
       </c>
-      <c r="D21" s="33" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>内径 4 mm；外径 7 mm；厚 0.3 mm</t>
         </is>
       </c>
-      <c r="E21" s="33" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>POM</t>
         </is>
       </c>
-      <c r="F21" s="32" t="n">
+      <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="32" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H21" s="33" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>下单选 4*7*0.3；最小包装为 500 个。</t>
         </is>
       </c>
-      <c r="I21" s="32" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J21" s="34" t="inlineStr">
+      <c r="J21" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mXao0V9CyJaiyk?tk=JJL4T3upc49</t>
         </is>
       </c>
-      <c r="K21" s="33" t="n"/>
-      <c r="L21" s="33" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>已核验：在售；规格匹配，包装数大于需求。</t>
         </is>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
-      <c r="A22" s="32" t="n">
+      <c r="A22" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="33" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C22" s="33" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>螺丝</t>
         </is>
       </c>
-      <c r="D22" s="33" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>M2 x 10 mm</t>
         </is>
       </c>
-      <c r="E22" s="33" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>TA2 钛合金</t>
         </is>
       </c>
-      <c r="F22" s="32" t="n">
+      <c r="F22" t="n">
         <v>10</v>
       </c>
-      <c r="G22" s="32" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H22" s="33" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>下单选 M2*10【10只】。</t>
         </is>
       </c>
-      <c r="I22" s="32" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J22" s="34" t="inlineStr">
+      <c r="J22" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8k9HQxnIM9sNRd8?tk=gbwHT3uguuB</t>
         </is>
       </c>
-      <c r="K22" s="33" t="n"/>
-      <c r="L22" s="33" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>已核验：在售、有货；包装数匹配。</t>
         </is>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="32" t="n">
+      <c r="A23" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="33" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C23" s="33" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>螺丝</t>
         </is>
       </c>
-      <c r="D23" s="33" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>M2 x 3 mm</t>
         </is>
       </c>
-      <c r="E23" s="33" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>TA2 钛合金</t>
         </is>
       </c>
-      <c r="F23" s="32" t="n">
+      <c r="F23" t="n">
         <v>10</v>
       </c>
-      <c r="G23" s="32" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H23" s="33" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>下单选 M2*3【10只】。</t>
         </is>
       </c>
-      <c r="I23" s="32" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J23" s="34" t="inlineStr">
+      <c r="J23" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8k9HQxnIM9sNRd8?tk=gbwHT3uguuB</t>
         </is>
       </c>
-      <c r="K23" s="33" t="n"/>
-      <c r="L23" s="33" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>已核验：在售、有货；包装数匹配。</t>
         </is>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="32" t="n">
+      <c r="A24" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="33" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C24" s="33" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>螺丝</t>
         </is>
       </c>
-      <c r="D24" s="33" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>M2 x 4 mm</t>
         </is>
       </c>
-      <c r="E24" s="33" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>TA2 钛合金</t>
         </is>
       </c>
-      <c r="F24" s="32" t="n">
+      <c r="F24" t="n">
         <v>10</v>
       </c>
-      <c r="G24" s="32" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H24" s="33" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>下单选 M2*4【10只】。</t>
         </is>
       </c>
-      <c r="I24" s="32" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J24" s="34" t="inlineStr">
+      <c r="J24" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8k9HQxnIM9sNRd8?tk=gbwHT3uguuB</t>
         </is>
       </c>
-      <c r="K24" s="33" t="n"/>
-      <c r="L24" s="33" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>已核验：在售、有货；包装数匹配。</t>
         </is>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1">
-      <c r="A25" s="32" t="n">
+      <c r="A25" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="33" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C25" s="33" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>螺丝</t>
         </is>
       </c>
-      <c r="D25" s="33" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>M2 x 5 mm</t>
         </is>
       </c>
-      <c r="E25" s="33" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>TA2 钛合金</t>
         </is>
       </c>
-      <c r="F25" s="32" t="n">
+      <c r="F25" t="n">
         <v>10</v>
       </c>
-      <c r="G25" s="32" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H25" s="33" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>下单选 M2*5【10只】。</t>
         </is>
       </c>
-      <c r="I25" s="32" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J25" s="34" t="inlineStr">
+      <c r="J25" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8k9HQxnIM9sNRd8?tk=gbwHT3uguuB</t>
         </is>
       </c>
-      <c r="K25" s="33" t="n"/>
-      <c r="L25" s="33" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>已核验：在售、有货；包装数匹配。</t>
         </is>
       </c>
     </row>
     <row r="26" ht="42" customHeight="1">
-      <c r="A26" s="32" t="n">
+      <c r="A26" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="33" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>螺丝</t>
         </is>
       </c>
-      <c r="D26" s="33" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>M2 x 3 mm</t>
         </is>
       </c>
-      <c r="E26" s="33" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>碳钢</t>
         </is>
       </c>
-      <c r="F26" s="32" t="n">
+      <c r="F26" t="n">
         <v>100</v>
       </c>
-      <c r="G26" s="32" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H26" s="33" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>按 M2 x 3 mm 处理</t>
         </is>
       </c>
-      <c r="I26" s="32" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J26" s="34" t="inlineStr">
+      <c r="J26" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8PkU8AL21aKIX46?tk=FnisT3uELki</t>
         </is>
       </c>
-      <c r="K26" s="33" t="n"/>
-      <c r="L26" s="33" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>已核验：在售；选 M2*3（100 个装）。</t>
         </is>
       </c>
     </row>
     <row r="27" ht="42" customHeight="1">
-      <c r="A27" s="32" t="n">
+      <c r="A27" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="33" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C27" s="33" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>螺丝</t>
         </is>
       </c>
-      <c r="D27" s="33" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>M2 x 4 mm</t>
         </is>
       </c>
-      <c r="E27" s="33" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>碳钢</t>
         </is>
       </c>
-      <c r="F27" s="32" t="n">
+      <c r="F27" t="n">
         <v>100</v>
       </c>
-      <c r="G27" s="32" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H27" s="33" t="n"/>
-      <c r="I27" s="32" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J27" s="34" t="inlineStr">
+      <c r="J27" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8PkU8AL21aKIX46?tk=FnisT3uELki</t>
         </is>
       </c>
-      <c r="K27" s="33" t="n"/>
-      <c r="L27" s="33" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>已核验：在售；选 M2*4（100 个装）。</t>
         </is>
       </c>
     </row>
     <row r="28" ht="42" customHeight="1">
-      <c r="A28" s="32" t="n">
+      <c r="A28" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="33" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C28" s="33" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>半圆头内六角螺丝</t>
         </is>
       </c>
-      <c r="D28" s="33" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>M2 x 6 mm</t>
         </is>
       </c>
-      <c r="E28" s="33" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>铝合金</t>
         </is>
       </c>
-      <c r="F28" s="32" t="n">
+      <c r="F28" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="32" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H28" s="33" t="n"/>
-      <c r="I28" s="32" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J28" s="34" t="inlineStr">
+      <c r="J28" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mXeBmJXwCWEfkR?tk=2YwvT3uFI8e</t>
         </is>
       </c>
-      <c r="K28" s="33" t="n"/>
-      <c r="L28" s="33" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>已核验：在售；选 M2*6，商品为 2 个装。</t>
         </is>
       </c>
     </row>
     <row r="29" ht="42" customHeight="1">
-      <c r="A29" s="32" t="n">
+      <c r="A29" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="33" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C29" s="33" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>铝柱</t>
         </is>
       </c>
-      <c r="D29" s="33" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>M2 x 3.5 mm</t>
         </is>
       </c>
-      <c r="E29" s="33" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>铝合金</t>
         </is>
       </c>
-      <c r="F29" s="32" t="n">
+      <c r="F29" t="n">
         <v>10</v>
       </c>
-      <c r="G29" s="32" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H29" s="33" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>下单选 M2*3.5-D=3.5MM（10支）。</t>
         </is>
       </c>
-      <c r="I29" s="32" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J29" s="34" t="inlineStr">
+      <c r="J29" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mcJbt6WjCP0JSy?tk=iGsAT3uTzSu</t>
         </is>
       </c>
-      <c r="K29" s="33" t="n"/>
-      <c r="L29" s="33" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>已核验：在售、有货；规格与 10 支包装匹配。</t>
         </is>
       </c>
     </row>
     <row r="30" ht="42" customHeight="1">
-      <c r="A30" s="32" t="n">
+      <c r="A30" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="33" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>铝柱</t>
         </is>
       </c>
-      <c r="D30" s="33" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>M2 x 5 mm</t>
         </is>
       </c>
-      <c r="E30" s="33" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>铝合金</t>
         </is>
       </c>
-      <c r="F30" s="32" t="n">
+      <c r="F30" t="n">
         <v>10</v>
       </c>
-      <c r="G30" s="32" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H30" s="33" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>下单选 M2*5-D=3.5MM（10支）。</t>
         </is>
       </c>
-      <c r="I30" s="32" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J30" s="34" t="inlineStr">
+      <c r="J30" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mcJbt6WjCP0JSy?tk=iGsAT3uTzSu</t>
         </is>
       </c>
-      <c r="K30" s="33" t="n"/>
-      <c r="L30" s="33" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>已核验：在售、有货；规格与 10 支包装匹配。</t>
         </is>
       </c>
     </row>
     <row r="31" ht="42" customHeight="1">
-      <c r="A31" s="32" t="n">
+      <c r="A31" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="33" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C31" s="33" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>铝柱</t>
         </is>
       </c>
-      <c r="D31" s="33" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>M2 x 6.8 mm</t>
         </is>
       </c>
-      <c r="E31" s="33" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>铝合金</t>
         </is>
       </c>
-      <c r="F31" s="32" t="n">
+      <c r="F31" t="n">
         <v>10</v>
       </c>
-      <c r="G31" s="32" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H31" s="33" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>下单选 M2*6.8-D=3.5MM（10支）。</t>
         </is>
       </c>
-      <c r="I31" s="32" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J31" s="34" t="inlineStr">
+      <c r="J31" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mcJbt6WjCP0JSy?tk=iGsAT3uTzSu</t>
         </is>
       </c>
-      <c r="K31" s="33" t="n"/>
-      <c r="L31" s="33" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>已核验：在售、有货；规格与 10 支包装匹配。</t>
         </is>
       </c>
     </row>
     <row r="32" ht="42" customHeight="1">
-      <c r="A32" s="32" t="n">
+      <c r="A32" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="33" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>紧固件</t>
         </is>
       </c>
-      <c r="C32" s="33" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>铝柱</t>
         </is>
       </c>
-      <c r="D32" s="33" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>M2.5 x 15 mm</t>
         </is>
       </c>
-      <c r="E32" s="33" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>铝合金</t>
         </is>
       </c>
-      <c r="F32" s="32" t="n">
+      <c r="F32" t="n">
         <v>10</v>
       </c>
-      <c r="G32" s="32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H32" s="33" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>下单选 M2.5x15（D4），10 支。</t>
         </is>
       </c>
-      <c r="I32" s="32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J32" s="34" t="inlineStr">
+      <c r="J32" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8k9GsYJvXbqWoei?tk=fEgjT3uh7nR</t>
         </is>
       </c>
-      <c r="K32" s="33" t="n"/>
-      <c r="L32" s="33" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>已核验：在售、有货；规格与 10 支包装匹配。</t>
         </is>
       </c>
     </row>
     <row r="33" ht="42" customHeight="1">
-      <c r="A33" s="35" t="n">
+      <c r="A33" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="36" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>减振</t>
         </is>
       </c>
-      <c r="C33" s="36" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>橡胶垫片</t>
         </is>
       </c>
-      <c r="D33" s="36" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>内径 2 mm；外径 5 mm；厚 1.5 mm</t>
         </is>
       </c>
-      <c r="E33" s="36" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>橡胶</t>
         </is>
       </c>
-      <c r="F33" s="35" t="n">
+      <c r="F33" t="n">
         <v>20</v>
       </c>
-      <c r="G33" s="35" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H33" s="36" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>下单选 2*5*1.5（20只）。</t>
         </is>
       </c>
-      <c r="I33" s="35" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J33" s="31" t="inlineStr">
+      <c r="J33" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8lpP91xfSjr0gZL?tk=kItUT3uptxv</t>
         </is>
       </c>
-      <c r="K33" s="36" t="n"/>
-      <c r="L33" s="36" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>已核验：在售、有货；规格与数量匹配。</t>
         </is>
       </c>
     </row>
     <row r="34" ht="42" customHeight="1">
-      <c r="A34" s="37" t="n">
+      <c r="A34" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="38" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>减振</t>
         </is>
       </c>
-      <c r="C34" s="38" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>聚氨酯海绵</t>
         </is>
       </c>
-      <c r="D34" s="38" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>待按安装尺寸裁切</t>
         </is>
       </c>
-      <c r="E34" s="38" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>聚氨酯</t>
         </is>
       </c>
-      <c r="F34" s="37" t="n">
+      <c r="F34" t="n">
         <v>1</v>
       </c>
-      <c r="G34" s="37" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H34" s="38" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>用于 PCB/IMU 减振</t>
         </is>
       </c>
-      <c r="I34" s="37" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J34" s="34" t="inlineStr">
+      <c r="J34" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8lpkXIzQXcTAgRS?tk=cteeT3uL62O</t>
         </is>
       </c>
-      <c r="K34" s="38" t="n"/>
-      <c r="L34" s="38" t="inlineStr"/>
     </row>
     <row r="35" ht="42" customHeight="1">
-      <c r="A35" s="39" t="n">
+      <c r="A35" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="40" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>传动</t>
         </is>
       </c>
-      <c r="C35" s="40" t="inlineStr">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>编码器径向充磁磁铁</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>圆形径向充磁；尺寸待按编码器型号确认</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>N35 钕铁硼，镍镀层</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>4</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>四轮编码器各 1 个；安装磁铁与编码器的实际间距约 1 mm。</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J35" s="67" t="inlineStr">
+        <is>
+          <t>https://e.tb.cn/h.8mBtW10luYOM3fO?tk=Exr9TeJeSW9</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>已核验：在售、有货；可选 10/20/50/100 个装。下单前必须确认直径和厚度，勿按起价直接购买。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>传动</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>轴承</t>
         </is>
       </c>
-      <c r="D35" s="40" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>内径 4 mm；外径 11 mm；厚 4 mm</t>
         </is>
       </c>
-      <c r="E35" s="40" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>PEEK 或同尺寸替代</t>
         </is>
       </c>
-      <c r="F35" s="39" t="n">
+      <c r="F36" t="n">
         <v>8</v>
       </c>
-      <c r="G35" s="39" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H35" s="40" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>轮毂轴承；下单选 PEEK694（内径 4 mm、外径 11 mm、厚 4 mm）。</t>
         </is>
       </c>
-      <c r="I35" s="39" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J35" s="31" t="inlineStr">
+      <c r="J36" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mcxILEdGMrRZHv?tk=NkVrT3uOocV</t>
         </is>
       </c>
-      <c r="K35" s="40" t="n"/>
-      <c r="L35" s="40" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>已核验：在售、有货；规格 PEEK694 完全匹配。</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="42" customHeight="1">
-      <c r="A36" s="41" t="n">
-        <v>32</v>
-      </c>
-      <c r="B36" s="42" t="inlineStr">
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>传动</t>
         </is>
       </c>
-      <c r="C36" s="42" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>黄铜齿轮</t>
         </is>
       </c>
-      <c r="D36" s="42" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>1:5 减速比配套；0.5 模，10 齿</t>
         </is>
       </c>
-      <c r="E36" s="42" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>黄铜</t>
         </is>
       </c>
-      <c r="F36" s="41" t="n">
+      <c r="F37" t="n">
         <v>2</v>
       </c>
-      <c r="G36" s="41" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H36" s="42" t="n"/>
-      <c r="I36" s="41" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J36" s="34" t="inlineStr">
+      <c r="J37" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mXUdcSt3XmXSnl?tk=1mKJT3uEBDK</t>
         </is>
       </c>
-      <c r="K36" s="42" t="n"/>
-      <c r="L36" s="42" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>已核验：在售；选 10 齿。轴孔有 1.45/1.95/2.25/2.95 mm，按电机轴径选择。</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="42" customHeight="1">
-      <c r="A37" s="41" t="n">
-        <v>33</v>
-      </c>
-      <c r="B37" s="42" t="inlineStr">
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>传动</t>
         </is>
       </c>
-      <c r="C37" s="42" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>黄铜齿轮（1:8.5 配套）</t>
         </is>
       </c>
-      <c r="D37" s="42" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>1:8.5 减速比配套；0.4 模，8 齿</t>
         </is>
       </c>
-      <c r="E37" s="42" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>黄铜</t>
         </is>
       </c>
-      <c r="F37" s="41" t="n">
+      <c r="F38" t="n">
         <v>2</v>
       </c>
-      <c r="G37" s="41" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H37" s="42" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>与 1:5 的 0.5 模 10 齿齿轮二选一。</t>
         </is>
       </c>
-      <c r="I37" s="41" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J37" s="34" t="inlineStr">
+      <c r="J38" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mXU98qGpzvzAW9?tk=36ViT3uwCD4</t>
         </is>
       </c>
-      <c r="K37" s="42" t="inlineStr"/>
-      <c r="L37" s="42" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>已核验：在售；选 8 齿、外径 4 mm、孔 1.48 mm、厚 4 mm。</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="42" customHeight="1">
-      <c r="A38" s="43" t="n">
-        <v>34</v>
-      </c>
-      <c r="B38" s="44" t="inlineStr">
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>轮胎</t>
         </is>
       </c>
-      <c r="C38" s="44" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>龙邱 N 车模胎皮</t>
         </is>
       </c>
-      <c r="D38" s="44" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>龙邱 N 车模规格</t>
         </is>
       </c>
-      <c r="E38" s="44" t="n"/>
-      <c r="F38" s="43" t="n">
+      <c r="F39" t="n">
         <v>4</v>
       </c>
-      <c r="G38" s="43" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="H38" s="44" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>下单选“闪电鼠-N超软硅胶轮胎”，数量 4。</t>
         </is>
       </c>
-      <c r="I38" s="43" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J38" s="31" t="inlineStr">
+      <c r="J39" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8P9t6THlsmDb02D?tk=3HiqT3u72p8</t>
         </is>
       </c>
-      <c r="K38" s="44" t="n"/>
-      <c r="L38" s="44" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>已核验：预售，约 5 天发货。</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="42" customHeight="1">
-      <c r="A39" s="45" t="n">
-        <v>35</v>
-      </c>
-      <c r="B39" s="46" t="inlineStr">
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" t="inlineStr">
         <is>
           <t>行进</t>
         </is>
       </c>
-      <c r="C39" s="46" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>无刷电机</t>
         </is>
       </c>
-      <c r="D39" s="46" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>T-Motor F1404，3800 KV</t>
         </is>
       </c>
-      <c r="E39" s="46" t="n"/>
-      <c r="F39" s="45" t="n">
+      <c r="F40" t="n">
         <v>2</v>
       </c>
-      <c r="G39" s="45" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H39" s="46" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>行进电机；下单选 3800KV、一颗装。</t>
         </is>
       </c>
-      <c r="I39" s="45" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J39" s="31" t="inlineStr">
+      <c r="J40" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mX8okkLmuej62t?tk=hs43T3F0tV7</t>
         </is>
       </c>
-      <c r="K39" s="46" t="n"/>
-      <c r="L39" s="46" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>已核验：在售、有货。</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="42" customHeight="1">
-      <c r="A40" s="47" t="n">
-        <v>36</v>
-      </c>
-      <c r="B40" s="48" t="inlineStr">
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>负压</t>
         </is>
       </c>
-      <c r="C40" s="48" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>无刷电机</t>
         </is>
       </c>
-      <c r="D40" s="48" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>致盈动力 GTS V2 1202.5，6000 KV</t>
         </is>
       </c>
-      <c r="E40" s="48" t="n"/>
-      <c r="F40" s="47" t="n">
+      <c r="F41" t="n">
         <v>1</v>
       </c>
-      <c r="G40" s="47" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>颗</t>
         </is>
       </c>
-      <c r="H40" s="48" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>负压电机；下单选 6000KV【3-4S】一个装。</t>
         </is>
       </c>
-      <c r="I40" s="47" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J40" s="31" t="inlineStr">
+      <c r="J41" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mXRO5DbPoWJfw9?tk=By03T3F0om4</t>
         </is>
       </c>
-      <c r="K40" s="48" t="n"/>
-      <c r="L40" s="48" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>已核验：在售、有货；商品型号为 GTS V2 1202.5。</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="42" customHeight="1">
-      <c r="A41" s="49" t="n">
-        <v>37</v>
-      </c>
-      <c r="B41" s="50" t="inlineStr">
+    <row r="42" ht="42" customHeight="1">
+      <c r="A42" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>负压</t>
         </is>
       </c>
-      <c r="C41" s="50" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>负压膜</t>
         </is>
       </c>
-      <c r="D41" s="50" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>晨光书皮</t>
         </is>
       </c>
-      <c r="E41" s="50" t="n"/>
-      <c r="F41" s="49" t="n">
+      <c r="F42" t="n">
         <v>1</v>
       </c>
-      <c r="G41" s="49" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H41" s="50" t="n"/>
-      <c r="I41" s="49" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J41" s="34" t="inlineStr">
+      <c r="J42" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mX0D4OeRIXlw04?tk=ocbqT3uqjSP</t>
         </is>
       </c>
-      <c r="K41" s="50" t="n"/>
-      <c r="L41" s="50" t="inlineStr"/>
-    </row>
-    <row r="42" ht="42" customHeight="1">
-      <c r="A42" s="49" t="n">
-        <v>38</v>
-      </c>
-      <c r="B42" s="50" t="inlineStr">
+    </row>
+    <row r="43" ht="42" customHeight="1">
+      <c r="A43" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>负压</t>
         </is>
       </c>
-      <c r="C42" s="50" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>风机</t>
         </is>
       </c>
-      <c r="D42" s="50" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>龙邱 1202.5 尼龙无刷离心风机</t>
         </is>
       </c>
-      <c r="E42" s="50" t="n"/>
-      <c r="F42" s="49" t="n">
+      <c r="F43" t="n">
         <v>1</v>
       </c>
-      <c r="G42" s="49" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>份</t>
         </is>
       </c>
-      <c r="H42" s="50" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>下单选“1202.5 尼龙无刷离心风机”，不要误选负压无刷电机。</t>
         </is>
       </c>
-      <c r="I42" s="49" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J42" s="34" t="inlineStr">
+      <c r="J43" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8PkSTi588UCBtaw?tk=dKFCT3uBW81</t>
         </is>
       </c>
-      <c r="K42" s="50" t="n"/>
-      <c r="L42" s="50" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>已核验：在售；同一链接同时售风机、电机和软膜。</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="42" customHeight="1">
-      <c r="A43" s="51" t="n">
-        <v>39</v>
-      </c>
-      <c r="B43" s="52" t="inlineStr">
+    <row r="44" ht="42" customHeight="1">
+      <c r="A44" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>粘接</t>
         </is>
       </c>
-      <c r="C43" s="52" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>双面胶</t>
         </is>
       </c>
-      <c r="D43" s="52" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>3M 9495</t>
         </is>
       </c>
-      <c r="E43" s="52" t="n"/>
-      <c r="F43" s="51" t="n">
+      <c r="F44" t="n">
         <v>1</v>
       </c>
-      <c r="G43" s="51" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>卷</t>
         </is>
       </c>
-      <c r="H43" s="52" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>用于贴负压</t>
         </is>
       </c>
-      <c r="I43" s="51" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J43" s="31" t="inlineStr">
+      <c r="J44" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8lp7YVn7C9ZhFWG?tk=GcDuT3ulg6z</t>
         </is>
       </c>
-      <c r="K43" s="52" t="n"/>
-      <c r="L43" s="52" t="inlineStr"/>
-    </row>
-    <row r="44" ht="42" customHeight="1">
-      <c r="A44" s="53" t="n">
-        <v>40</v>
-      </c>
-      <c r="B44" s="54" t="inlineStr">
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>粘接</t>
         </is>
       </c>
-      <c r="C44" s="54" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>双面胶</t>
         </is>
       </c>
-      <c r="D44" s="54" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>3M VHB</t>
         </is>
       </c>
-      <c r="E44" s="54" t="n"/>
-      <c r="F44" s="53" t="n">
+      <c r="F45" t="n">
         <v>1</v>
       </c>
-      <c r="G44" s="53" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>卷</t>
         </is>
       </c>
-      <c r="H44" s="54" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>用于需方便拆除的粘接部位</t>
         </is>
       </c>
-      <c r="I44" s="53" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="J44" s="34" t="inlineStr">
+      <c r="J45" s="67" t="inlineStr">
         <is>
           <t>https://e.tb.cn/h.8mcD9pQHB3meS3g?tk=mwmQT3ulk7c</t>
         </is>
       </c>
-      <c r="K44" s="54" t="n"/>
-      <c r="L44" s="54" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L44"/>
+  <autoFilter ref="A4:L45"/>
   <mergeCells count="3">
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="A2:L2"/>
@@ -3788,11 +3802,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3987,7 +4002,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="63" t="inlineStr">
         <is>
@@ -3996,7 +4010,7 @@
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="64" t="inlineStr">
+      <c r="A19" s="68" t="inlineStr">
         <is>
           <t>预计总开销：约 600 元，不含轴承。该数字是当前清单的粗略预算，不是报价或费用承诺；实际价格、运费、加工费和材料损耗会随渠道与版本变化。</t>
         </is>
@@ -4005,7 +4019,7 @@
       <c r="C19" s="66" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="64" t="inlineStr">
+      <c r="A20" s="68" t="inlineStr">
         <is>
           <t>其中：CNC 加工 + 碳板 + 3D 打印约 250 元出头；三颗电机约 250 元；零散紧固件、胶带、垫片、胎皮等物料约 100 多元。</t>
         </is>
@@ -4014,7 +4028,7 @@
       <c r="C20" s="66" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="64" t="inlineStr">
+      <c r="A21" s="68" t="inlineStr">
         <is>
           <t>本清单和机械资料仅用于设计参考与学习，不保证适配每一块场地、每一批材料或每种加工工艺，也不构成安全、性能或可制造性担保。</t>
         </is>
@@ -4023,7 +4037,7 @@
       <c r="C21" s="66" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="65" t="inlineStr">
+      <c r="A22" s="69" t="inlineStr">
         <is>
           <t>如有经济压力，可以将底盘、传动、负压、传感器安装等拆分为多个模块自行设计和验证；欢迎参考设计思路，不建议完全机械复刻。</t>
         </is>
@@ -4032,7 +4046,7 @@
       <c r="C22" s="66" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="65" t="inlineStr">
+      <c r="A23" s="69" t="inlineStr">
         <is>
           <t>涉及高速电机、负压、刀具和 CNC/3D 打印加工时，请自行完成强度、干涉、电气和安全验证，并从低速、架空测试开始。</t>
         </is>

</xml_diff>